<commit_message>
Refactor data handling and reporting functions; update output file naming conventions
- Updated `read_data` function in `model_data.py` to correct handling capacity field names and ensure consistency in data extraction.
- Modified `write_results`, `write_dual`, `write_fleet`, and `write_objective_sensitivity` functions in `reporting.py` to include a `suffix` parameter for output file naming, allowing for versioned outputs.
- Added new dependencies in `requirements.txt` for PyYAML.
- Created new result files for dual prices, fleet capacity, shipments, and summary in the `results` directory with an "ALTERNATIVE" suffix.
- Updated visualization functions to support versioned output file names for network and solution maps.
</commit_message>
<xml_diff>
--- a/Data/Data DMO Project 1 ALTERNATIVE.xlsx
+++ b/Data/Data DMO Project 1 ALTERNATIVE.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jonathan/Desktop/Masters/Decision Making and Optimization/Assignments/DMO Assignment Project 1/DMO-Project-1-Baseline-Problem---Group-11/Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DC1D778A-61BD-4643-A3FD-FB967FFF088C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E60A11A-2734-B04B-BEAD-4D5D5ABCF2E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="17140" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,17 +37,11 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="154" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="38">
   <si>
     <t>centre_id</t>
   </si>
   <si>
-    <t>centre_name</t>
-  </si>
-  <si>
-    <t>handling_capacity_equiv</t>
-  </si>
-  <si>
     <t>x_km</t>
   </si>
   <si>
@@ -57,75 +51,33 @@
     <t>L1</t>
   </si>
   <si>
-    <t>North Hub</t>
-  </si>
-  <si>
     <t>L2</t>
   </si>
   <si>
-    <t>Central Hub</t>
-  </si>
-  <si>
     <t>L3</t>
   </si>
   <si>
-    <t>South Hub</t>
-  </si>
-  <si>
     <t>region_id</t>
   </si>
   <si>
-    <t>region_name</t>
-  </si>
-  <si>
-    <t>severity</t>
-  </si>
-  <si>
     <t>R1</t>
   </si>
   <si>
-    <t>North Coast</t>
-  </si>
-  <si>
-    <t>High</t>
-  </si>
-  <si>
     <t>R2</t>
   </si>
   <si>
-    <t>North Inland</t>
-  </si>
-  <si>
-    <t>Medium</t>
-  </si>
-  <si>
     <t>R3</t>
   </si>
   <si>
-    <t>Central City</t>
-  </si>
-  <si>
-    <t>Critical</t>
-  </si>
-  <si>
     <t>R4</t>
   </si>
   <si>
-    <t>East Valley</t>
-  </si>
-  <si>
     <t>R5</t>
   </si>
   <si>
-    <t>South Coast</t>
-  </si>
-  <si>
     <t>R6</t>
   </si>
   <si>
-    <t>Mountain District</t>
-  </si>
-  <si>
     <t>resource_id</t>
   </si>
   <si>
@@ -135,48 +87,30 @@
     <t>unit</t>
   </si>
   <si>
-    <t>handling_equiv_per_unit</t>
-  </si>
-  <si>
     <t>transport_rate_eur_per_unit_km</t>
   </si>
   <si>
-    <t>K1</t>
-  </si>
-  <si>
     <t>Drinking water</t>
   </si>
   <si>
     <t>case</t>
   </si>
   <si>
-    <t>K2</t>
-  </si>
-  <si>
     <t>Food parcels</t>
   </si>
   <si>
     <t>parcel</t>
   </si>
   <si>
-    <t>K3</t>
-  </si>
-  <si>
     <t>Medical kits</t>
   </si>
   <si>
     <t>kit</t>
   </si>
   <si>
-    <t>K4</t>
-  </si>
-  <si>
     <t>Shelter kits</t>
   </si>
   <si>
-    <t>K5</t>
-  </si>
-  <si>
     <t>Hygiene kits</t>
   </si>
   <si>
@@ -196,6 +130,27 @@
   </si>
   <si>
     <t>cargo_volume_per_unit</t>
+  </si>
+  <si>
+    <t>handling_capacity</t>
+  </si>
+  <si>
+    <t>V1</t>
+  </si>
+  <si>
+    <t>V2</t>
+  </si>
+  <si>
+    <t>V3</t>
+  </si>
+  <si>
+    <t>V4</t>
+  </si>
+  <si>
+    <t>V5</t>
+  </si>
+  <si>
+    <t>handling_per_unit</t>
   </si>
 </sst>
 </file>
@@ -206,7 +161,7 @@
     <numFmt numFmtId="164" formatCode="0.0"/>
     <numFmt numFmtId="165" formatCode="0.000"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <sz val="11"/>
       <name val="Carlito"/>
@@ -217,8 +172,13 @@
       <color rgb="FFFFFFFF"/>
       <name val="Carlito"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Carlito"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -235,8 +195,14 @@
         <fgColor rgb="FF17365D"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD9D9D9"/>
+        <bgColor rgb="FFD9D9D9"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -244,11 +210,24 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -256,6 +235,8 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -274,17 +255,16 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="CentresTable" displayName="CentresTable" ref="A1:H4" totalsRowShown="0">
-  <tableColumns count="8">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="CentresTable" displayName="CentresTable" ref="A1:G4" totalsRowShown="0">
+  <tableColumns count="7">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="centre_id"/>
-    <tableColumn id="7" xr3:uid="{D5C64500-EB07-0B4A-9801-B2C1420AB480}" name="centre_name"/>
-    <tableColumn id="8" xr3:uid="{16409BF7-3049-0D48-97A9-40830532605C}" name="handling_capacity_equiv"/>
+    <tableColumn id="8" xr3:uid="{16409BF7-3049-0D48-97A9-40830532605C}" name="handling_capacity"/>
     <tableColumn id="9" xr3:uid="{BB2DCDBB-72B5-8842-AFDF-52A5D5069BE3}" name="x_km"/>
     <tableColumn id="10" xr3:uid="{D1B0641E-2DF4-F041-9F9F-96250AB145FB}" name="y_km"/>
     <tableColumn id="11" xr3:uid="{FC9E1F8E-0C42-A644-8631-1D914F678F1B}" name="trucks_available"/>
     <tableColumn id="12" xr3:uid="{83FAE226-9838-944E-B788-695EC3661FF8}" name="truck_capacity"/>
     <tableColumn id="13" xr3:uid="{B7373347-03B3-CA40-A420-C88316248B92}" name="fleet_capacity">
-      <calculatedColumnFormula>F2*G2</calculatedColumnFormula>
+      <calculatedColumnFormula>E2*F2</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -292,11 +272,9 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="RegionsTable" displayName="RegionsTable" ref="A1:E7" totalsRowShown="0">
-  <tableColumns count="5">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="RegionsTable" displayName="RegionsTable" ref="A1:C7" totalsRowShown="0">
+  <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0100-000001000000}" name="region_id"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0100-000002000000}" name="region_name"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0100-000003000000}" name="severity"/>
     <tableColumn id="4" xr3:uid="{00000000-0010-0000-0100-000004000000}" name="x_km"/>
     <tableColumn id="5" xr3:uid="{00000000-0010-0000-0100-000005000000}" name="y_km"/>
   </tableColumns>
@@ -310,7 +288,7 @@
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0200-000001000000}" name="resource_id"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0200-000002000000}" name="resource_name"/>
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0200-000003000000}" name="unit"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0200-000004000000}" name="handling_equiv_per_unit"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0200-000004000000}" name="handling_per_unit"/>
     <tableColumn id="5" xr3:uid="{00000000-0010-0000-0200-000005000000}" name="transport_rate_eur_per_unit_km"/>
     <tableColumn id="6" xr3:uid="{1CBDFA77-EA0B-6D4F-BB9B-8EE2436F0E55}" name="cargo_volume_per_unit"/>
   </tableColumns>
@@ -535,124 +513,111 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:G4"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="9.33203125" customWidth="1"/>
-    <col min="2" max="2" width="12.5" customWidth="1"/>
-    <col min="3" max="3" width="23.5" customWidth="1"/>
-    <col min="4" max="5" width="5.83203125" customWidth="1"/>
-    <col min="6" max="6" width="15.33203125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="13.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="23.5" customWidth="1"/>
+    <col min="3" max="4" width="5.83203125" customWidth="1"/>
+    <col min="5" max="5" width="15.33203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="30" customHeight="1">
+    <row r="1" spans="1:7" ht="30" customHeight="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="G1" s="4" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" ht="20" customHeight="1">
+      <c r="A2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="4" t="s">
-        <v>49</v>
-      </c>
-      <c r="G1" s="4" t="s">
-        <v>50</v>
-      </c>
-      <c r="H1" s="4" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" ht="20" customHeight="1">
-      <c r="A2" t="s">
-        <v>5</v>
-      </c>
-      <c r="B2" t="s">
-        <v>6</v>
-      </c>
-      <c r="C2">
+      <c r="B2">
         <f>684-59.2</f>
         <v>624.79999999999995</v>
       </c>
+      <c r="C2">
+        <v>20</v>
+      </c>
       <c r="D2">
-        <v>20</v>
+        <v>300</v>
       </c>
       <c r="E2">
-        <v>300</v>
+        <v>9</v>
       </c>
       <c r="F2">
-        <v>9</v>
+        <v>30</v>
       </c>
       <c r="G2">
-        <v>30</v>
-      </c>
-      <c r="H2">
         <f>270-42.6</f>
         <v>227.4</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="20" customHeight="1">
+    <row r="3" spans="1:7" ht="20" customHeight="1">
       <c r="A3" t="s">
-        <v>7</v>
-      </c>
-      <c r="B3" t="s">
-        <v>8</v>
-      </c>
-      <c r="C3">
+        <v>4</v>
+      </c>
+      <c r="B3">
         <f>790+59.2+40.8</f>
         <v>890</v>
       </c>
+      <c r="C3">
+        <v>65</v>
+      </c>
       <c r="D3">
-        <v>65</v>
+        <v>160</v>
       </c>
       <c r="E3">
-        <v>160</v>
+        <v>8</v>
       </c>
       <c r="F3">
-        <v>8</v>
+        <v>30</v>
       </c>
       <c r="G3">
-        <v>30</v>
-      </c>
-      <c r="H3">
         <f>240+38.5+42.6</f>
         <v>321.10000000000002</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="20" customHeight="1">
+    <row r="4" spans="1:7" ht="20" customHeight="1">
       <c r="A4" t="s">
-        <v>9</v>
-      </c>
-      <c r="B4" t="s">
-        <v>10</v>
-      </c>
-      <c r="C4">
+        <v>5</v>
+      </c>
+      <c r="B4">
         <f>740-40.8</f>
         <v>699.2</v>
       </c>
+      <c r="C4">
+        <v>65</v>
+      </c>
       <c r="D4">
-        <v>65</v>
+        <v>15</v>
       </c>
       <c r="E4">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="F4">
-        <v>9</v>
+        <v>30</v>
       </c>
       <c r="G4">
-        <v>30</v>
-      </c>
-      <c r="H4">
         <f>270-38.5</f>
         <v>231.5</v>
       </c>
@@ -667,131 +632,87 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:C7"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="15" customWidth="1"/>
-    <col min="2" max="2" width="24" customWidth="1"/>
-    <col min="3" max="3" width="12.5" customWidth="1"/>
-    <col min="4" max="5" width="12" customWidth="1"/>
+    <col min="2" max="3" width="12" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="28" customHeight="1">
+    <row r="1" spans="1:3" ht="28" customHeight="1">
       <c r="A1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" ht="20" customHeight="1">
+      <c r="A2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B2">
+        <v>15</v>
+      </c>
+      <c r="C2">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" ht="20" customHeight="1">
+      <c r="A3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B3">
+        <v>90</v>
+      </c>
+      <c r="C3">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" ht="20" customHeight="1">
+      <c r="A4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4">
+        <v>67</v>
+      </c>
+      <c r="C4">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" ht="20" customHeight="1">
+      <c r="A5" t="s">
+        <v>10</v>
+      </c>
+      <c r="B5">
+        <v>135</v>
+      </c>
+      <c r="C5">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" ht="20" customHeight="1">
+      <c r="A6" t="s">
         <v>11</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B6">
+        <v>105</v>
+      </c>
+      <c r="C6">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" ht="20" customHeight="1">
+      <c r="A7" t="s">
         <v>12</v>
       </c>
-      <c r="C1" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" ht="20" customHeight="1">
-      <c r="A2" t="s">
-        <v>14</v>
-      </c>
-      <c r="B2" t="s">
-        <v>15</v>
-      </c>
-      <c r="C2" t="s">
-        <v>16</v>
-      </c>
-      <c r="D2">
-        <v>15</v>
-      </c>
-      <c r="E2">
-        <v>270</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" ht="20" customHeight="1">
-      <c r="A3" t="s">
-        <v>17</v>
-      </c>
-      <c r="B3" t="s">
-        <v>18</v>
-      </c>
-      <c r="C3" t="s">
-        <v>19</v>
-      </c>
-      <c r="D3">
-        <v>90</v>
-      </c>
-      <c r="E3">
-        <v>245</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" ht="20" customHeight="1">
-      <c r="A4" t="s">
-        <v>20</v>
-      </c>
-      <c r="B4" t="s">
-        <v>21</v>
-      </c>
-      <c r="C4" t="s">
+      <c r="B7">
         <v>22</v>
       </c>
-      <c r="D4">
-        <v>67</v>
-      </c>
-      <c r="E4">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" ht="20" customHeight="1">
-      <c r="A5" t="s">
-        <v>23</v>
-      </c>
-      <c r="B5" t="s">
-        <v>24</v>
-      </c>
-      <c r="C5" t="s">
-        <v>16</v>
-      </c>
-      <c r="D5">
-        <v>135</v>
-      </c>
-      <c r="E5">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" ht="20" customHeight="1">
-      <c r="A6" t="s">
-        <v>25</v>
-      </c>
-      <c r="B6" t="s">
-        <v>26</v>
-      </c>
-      <c r="C6" t="s">
-        <v>19</v>
-      </c>
-      <c r="D6">
-        <v>105</v>
-      </c>
-      <c r="E6">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" ht="20" customHeight="1">
-      <c r="A7" t="s">
-        <v>27</v>
-      </c>
-      <c r="B7" t="s">
-        <v>28</v>
-      </c>
-      <c r="C7" t="s">
-        <v>22</v>
-      </c>
-      <c r="D7">
-        <v>22</v>
-      </c>
-      <c r="E7">
+      <c r="C7">
         <v>80</v>
       </c>
     </row>
@@ -818,33 +739,33 @@
   <sheetData>
     <row r="1" spans="1:6" ht="30" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>29</v>
+        <v>13</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="F1" s="4" t="s">
         <v>30</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="F1" s="4" t="s">
-        <v>52</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="20" customHeight="1">
       <c r="A2" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="B2" t="s">
-        <v>35</v>
+        <v>17</v>
       </c>
       <c r="C2" t="s">
-        <v>36</v>
+        <v>18</v>
       </c>
       <c r="D2" s="2">
         <v>1</v>
@@ -858,13 +779,13 @@
     </row>
     <row r="3" spans="1:6" ht="20" customHeight="1">
       <c r="A3" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="B3" t="s">
-        <v>38</v>
+        <v>19</v>
       </c>
       <c r="C3" t="s">
-        <v>39</v>
+        <v>20</v>
       </c>
       <c r="D3" s="2">
         <v>1.2</v>
@@ -878,13 +799,13 @@
     </row>
     <row r="4" spans="1:6" ht="20" customHeight="1">
       <c r="A4" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="B4" t="s">
-        <v>41</v>
+        <v>21</v>
       </c>
       <c r="C4" t="s">
-        <v>42</v>
+        <v>22</v>
       </c>
       <c r="D4" s="2">
         <v>0.6</v>
@@ -898,13 +819,13 @@
     </row>
     <row r="5" spans="1:6" ht="20" customHeight="1">
       <c r="A5" t="s">
-        <v>43</v>
+        <v>35</v>
       </c>
       <c r="B5" t="s">
-        <v>44</v>
+        <v>23</v>
       </c>
       <c r="C5" t="s">
-        <v>42</v>
+        <v>22</v>
       </c>
       <c r="D5" s="2">
         <v>3</v>
@@ -918,13 +839,13 @@
     </row>
     <row r="6" spans="1:6" ht="20" customHeight="1">
       <c r="A6" t="s">
-        <v>45</v>
+        <v>36</v>
       </c>
       <c r="B6" t="s">
-        <v>46</v>
+        <v>24</v>
       </c>
       <c r="C6" t="s">
-        <v>42</v>
+        <v>22</v>
       </c>
       <c r="D6" s="2">
         <v>0.8</v>
@@ -958,18 +879,18 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>29</v>
+        <v>13</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>47</v>
+        <v>25</v>
       </c>
     </row>
     <row r="2" spans="1:3" ht="20" customHeight="1">
       <c r="A2" t="s">
-        <v>5</v>
-      </c>
-      <c r="B2" t="s">
-        <v>34</v>
+        <v>3</v>
+      </c>
+      <c r="B2" s="5" t="s">
+        <v>32</v>
       </c>
       <c r="C2">
         <v>230</v>
@@ -977,10 +898,10 @@
     </row>
     <row r="3" spans="1:3" ht="20" customHeight="1">
       <c r="A3" t="s">
-        <v>5</v>
-      </c>
-      <c r="B3" t="s">
-        <v>37</v>
+        <v>3</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>33</v>
       </c>
       <c r="C3">
         <v>160</v>
@@ -988,10 +909,10 @@
     </row>
     <row r="4" spans="1:3" ht="20" customHeight="1">
       <c r="A4" t="s">
-        <v>5</v>
-      </c>
-      <c r="B4" t="s">
-        <v>40</v>
+        <v>3</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>34</v>
       </c>
       <c r="C4">
         <v>50</v>
@@ -999,10 +920,10 @@
     </row>
     <row r="5" spans="1:3" ht="20" customHeight="1">
       <c r="A5" t="s">
-        <v>5</v>
-      </c>
-      <c r="B5" t="s">
-        <v>43</v>
+        <v>3</v>
+      </c>
+      <c r="B5" s="6" t="s">
+        <v>35</v>
       </c>
       <c r="C5">
         <v>54</v>
@@ -1010,10 +931,10 @@
     </row>
     <row r="6" spans="1:3" ht="20" customHeight="1">
       <c r="A6" t="s">
-        <v>5</v>
-      </c>
-      <c r="B6" t="s">
-        <v>45</v>
+        <v>3</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>36</v>
       </c>
       <c r="C6">
         <v>132</v>
@@ -1021,10 +942,10 @@
     </row>
     <row r="7" spans="1:3" ht="20" customHeight="1">
       <c r="A7" t="s">
-        <v>7</v>
-      </c>
-      <c r="B7" t="s">
-        <v>34</v>
+        <v>4</v>
+      </c>
+      <c r="B7" s="5" t="s">
+        <v>32</v>
       </c>
       <c r="C7">
         <v>230</v>
@@ -1032,10 +953,10 @@
     </row>
     <row r="8" spans="1:3" ht="20" customHeight="1">
       <c r="A8" t="s">
-        <v>7</v>
-      </c>
-      <c r="B8" t="s">
-        <v>37</v>
+        <v>4</v>
+      </c>
+      <c r="B8" s="6" t="s">
+        <v>33</v>
       </c>
       <c r="C8">
         <v>200</v>
@@ -1043,10 +964,10 @@
     </row>
     <row r="9" spans="1:3" ht="20" customHeight="1">
       <c r="A9" t="s">
-        <v>7</v>
-      </c>
-      <c r="B9" t="s">
-        <v>40</v>
+        <v>4</v>
+      </c>
+      <c r="B9" s="5" t="s">
+        <v>34</v>
       </c>
       <c r="C9">
         <v>90</v>
@@ -1054,10 +975,10 @@
     </row>
     <row r="10" spans="1:3" ht="20" customHeight="1">
       <c r="A10" t="s">
-        <v>7</v>
-      </c>
-      <c r="B10" t="s">
-        <v>43</v>
+        <v>4</v>
+      </c>
+      <c r="B10" s="6" t="s">
+        <v>35</v>
       </c>
       <c r="C10">
         <v>65</v>
@@ -1065,10 +986,10 @@
     </row>
     <row r="11" spans="1:3" ht="20" customHeight="1">
       <c r="A11" t="s">
-        <v>7</v>
-      </c>
-      <c r="B11" t="s">
-        <v>45</v>
+        <v>4</v>
+      </c>
+      <c r="B11" s="5" t="s">
+        <v>36</v>
       </c>
       <c r="C11">
         <v>155</v>
@@ -1076,10 +997,10 @@
     </row>
     <row r="12" spans="1:3" ht="20" customHeight="1">
       <c r="A12" t="s">
-        <v>9</v>
-      </c>
-      <c r="B12" t="s">
-        <v>34</v>
+        <v>5</v>
+      </c>
+      <c r="B12" s="5" t="s">
+        <v>32</v>
       </c>
       <c r="C12">
         <v>205</v>
@@ -1087,10 +1008,10 @@
     </row>
     <row r="13" spans="1:3" ht="20" customHeight="1">
       <c r="A13" t="s">
-        <v>9</v>
-      </c>
-      <c r="B13" t="s">
-        <v>37</v>
+        <v>5</v>
+      </c>
+      <c r="B13" s="6" t="s">
+        <v>33</v>
       </c>
       <c r="C13">
         <v>170</v>
@@ -1098,10 +1019,10 @@
     </row>
     <row r="14" spans="1:3" ht="20" customHeight="1">
       <c r="A14" t="s">
-        <v>9</v>
-      </c>
-      <c r="B14" t="s">
-        <v>40</v>
+        <v>5</v>
+      </c>
+      <c r="B14" s="5" t="s">
+        <v>34</v>
       </c>
       <c r="C14">
         <v>55</v>
@@ -1109,10 +1030,10 @@
     </row>
     <row r="15" spans="1:3" ht="20" customHeight="1">
       <c r="A15" t="s">
-        <v>9</v>
-      </c>
-      <c r="B15" t="s">
-        <v>43</v>
+        <v>5</v>
+      </c>
+      <c r="B15" s="6" t="s">
+        <v>35</v>
       </c>
       <c r="C15">
         <v>50</v>
@@ -1120,10 +1041,10 @@
     </row>
     <row r="16" spans="1:3" ht="20" customHeight="1">
       <c r="A16" t="s">
-        <v>9</v>
-      </c>
-      <c r="B16" t="s">
-        <v>45</v>
+        <v>5</v>
+      </c>
+      <c r="B16" s="5" t="s">
+        <v>36</v>
       </c>
       <c r="C16">
         <v>135</v>
@@ -1148,21 +1069,21 @@
   <sheetData>
     <row r="1" spans="1:3" ht="28" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>29</v>
+        <v>13</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>48</v>
+        <v>26</v>
       </c>
     </row>
     <row r="2" spans="1:3" ht="20" customHeight="1">
       <c r="A2" t="s">
-        <v>14</v>
-      </c>
-      <c r="B2" t="s">
-        <v>34</v>
+        <v>7</v>
+      </c>
+      <c r="B2" s="5" t="s">
+        <v>32</v>
       </c>
       <c r="C2">
         <v>110</v>
@@ -1170,10 +1091,10 @@
     </row>
     <row r="3" spans="1:3" ht="20" customHeight="1">
       <c r="A3" t="s">
-        <v>14</v>
-      </c>
-      <c r="B3" t="s">
-        <v>37</v>
+        <v>7</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>33</v>
       </c>
       <c r="C3">
         <v>75</v>
@@ -1181,10 +1102,10 @@
     </row>
     <row r="4" spans="1:3" ht="20" customHeight="1">
       <c r="A4" t="s">
-        <v>14</v>
-      </c>
-      <c r="B4" t="s">
-        <v>40</v>
+        <v>7</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>34</v>
       </c>
       <c r="C4">
         <v>28</v>
@@ -1192,10 +1113,10 @@
     </row>
     <row r="5" spans="1:3" ht="20" customHeight="1">
       <c r="A5" t="s">
-        <v>14</v>
-      </c>
-      <c r="B5" t="s">
-        <v>43</v>
+        <v>7</v>
+      </c>
+      <c r="B5" s="6" t="s">
+        <v>35</v>
       </c>
       <c r="C5">
         <v>24</v>
@@ -1203,10 +1124,10 @@
     </row>
     <row r="6" spans="1:3" ht="20" customHeight="1">
       <c r="A6" t="s">
-        <v>14</v>
-      </c>
-      <c r="B6" t="s">
-        <v>45</v>
+        <v>7</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>36</v>
       </c>
       <c r="C6">
         <v>65</v>
@@ -1214,10 +1135,10 @@
     </row>
     <row r="7" spans="1:3" ht="20" customHeight="1">
       <c r="A7" t="s">
-        <v>17</v>
-      </c>
-      <c r="B7" t="s">
-        <v>34</v>
+        <v>8</v>
+      </c>
+      <c r="B7" s="5" t="s">
+        <v>32</v>
       </c>
       <c r="C7">
         <v>90</v>
@@ -1225,10 +1146,10 @@
     </row>
     <row r="8" spans="1:3" ht="20" customHeight="1">
       <c r="A8" t="s">
-        <v>17</v>
-      </c>
-      <c r="B8" t="s">
-        <v>37</v>
+        <v>8</v>
+      </c>
+      <c r="B8" s="6" t="s">
+        <v>33</v>
       </c>
       <c r="C8">
         <v>65</v>
@@ -1236,10 +1157,10 @@
     </row>
     <row r="9" spans="1:3" ht="20" customHeight="1">
       <c r="A9" t="s">
-        <v>17</v>
-      </c>
-      <c r="B9" t="s">
-        <v>40</v>
+        <v>8</v>
+      </c>
+      <c r="B9" s="5" t="s">
+        <v>34</v>
       </c>
       <c r="C9">
         <v>20</v>
@@ -1247,10 +1168,10 @@
     </row>
     <row r="10" spans="1:3" ht="20" customHeight="1">
       <c r="A10" t="s">
-        <v>17</v>
-      </c>
-      <c r="B10" t="s">
-        <v>43</v>
+        <v>8</v>
+      </c>
+      <c r="B10" s="6" t="s">
+        <v>35</v>
       </c>
       <c r="C10">
         <v>18</v>
@@ -1258,10 +1179,10 @@
     </row>
     <row r="11" spans="1:3" ht="20" customHeight="1">
       <c r="A11" t="s">
-        <v>17</v>
-      </c>
-      <c r="B11" t="s">
-        <v>45</v>
+        <v>8</v>
+      </c>
+      <c r="B11" s="5" t="s">
+        <v>36</v>
       </c>
       <c r="C11">
         <v>50</v>
@@ -1269,10 +1190,10 @@
     </row>
     <row r="12" spans="1:3" ht="20" customHeight="1">
       <c r="A12" t="s">
-        <v>20</v>
-      </c>
-      <c r="B12" t="s">
-        <v>34</v>
+        <v>9</v>
+      </c>
+      <c r="B12" s="5" t="s">
+        <v>32</v>
       </c>
       <c r="C12">
         <v>130</v>
@@ -1280,10 +1201,10 @@
     </row>
     <row r="13" spans="1:3" ht="20" customHeight="1">
       <c r="A13" t="s">
-        <v>20</v>
-      </c>
-      <c r="B13" t="s">
-        <v>37</v>
+        <v>9</v>
+      </c>
+      <c r="B13" s="6" t="s">
+        <v>33</v>
       </c>
       <c r="C13">
         <v>105</v>
@@ -1291,10 +1212,10 @@
     </row>
     <row r="14" spans="1:3" ht="20" customHeight="1">
       <c r="A14" t="s">
-        <v>20</v>
-      </c>
-      <c r="B14" t="s">
-        <v>40</v>
+        <v>9</v>
+      </c>
+      <c r="B14" s="5" t="s">
+        <v>34</v>
       </c>
       <c r="C14">
         <v>42</v>
@@ -1302,10 +1223,10 @@
     </row>
     <row r="15" spans="1:3" ht="20" customHeight="1">
       <c r="A15" t="s">
-        <v>20</v>
-      </c>
-      <c r="B15" t="s">
-        <v>43</v>
+        <v>9</v>
+      </c>
+      <c r="B15" s="6" t="s">
+        <v>35</v>
       </c>
       <c r="C15">
         <v>35</v>
@@ -1313,10 +1234,10 @@
     </row>
     <row r="16" spans="1:3" ht="20" customHeight="1">
       <c r="A16" t="s">
-        <v>20</v>
-      </c>
-      <c r="B16" t="s">
-        <v>45</v>
+        <v>9</v>
+      </c>
+      <c r="B16" s="5" t="s">
+        <v>36</v>
       </c>
       <c r="C16">
         <v>85</v>
@@ -1324,10 +1245,10 @@
     </row>
     <row r="17" spans="1:3" ht="20" customHeight="1">
       <c r="A17" t="s">
-        <v>23</v>
-      </c>
-      <c r="B17" t="s">
-        <v>34</v>
+        <v>10</v>
+      </c>
+      <c r="B17" s="5" t="s">
+        <v>32</v>
       </c>
       <c r="C17">
         <v>110</v>
@@ -1335,10 +1256,10 @@
     </row>
     <row r="18" spans="1:3" ht="20" customHeight="1">
       <c r="A18" t="s">
-        <v>23</v>
-      </c>
-      <c r="B18" t="s">
-        <v>37</v>
+        <v>10</v>
+      </c>
+      <c r="B18" s="6" t="s">
+        <v>33</v>
       </c>
       <c r="C18">
         <v>75</v>
@@ -1346,10 +1267,10 @@
     </row>
     <row r="19" spans="1:3" ht="20" customHeight="1">
       <c r="A19" t="s">
-        <v>23</v>
-      </c>
-      <c r="B19" t="s">
-        <v>40</v>
+        <v>10</v>
+      </c>
+      <c r="B19" s="5" t="s">
+        <v>34</v>
       </c>
       <c r="C19">
         <v>30</v>
@@ -1357,10 +1278,10 @@
     </row>
     <row r="20" spans="1:3" ht="20" customHeight="1">
       <c r="A20" t="s">
-        <v>23</v>
-      </c>
-      <c r="B20" t="s">
-        <v>43</v>
+        <v>10</v>
+      </c>
+      <c r="B20" s="6" t="s">
+        <v>35</v>
       </c>
       <c r="C20">
         <v>26</v>
@@ -1368,10 +1289,10 @@
     </row>
     <row r="21" spans="1:3" ht="20" customHeight="1">
       <c r="A21" t="s">
-        <v>23</v>
-      </c>
-      <c r="B21" t="s">
-        <v>45</v>
+        <v>10</v>
+      </c>
+      <c r="B21" s="5" t="s">
+        <v>36</v>
       </c>
       <c r="C21">
         <v>65</v>
@@ -1379,10 +1300,10 @@
     </row>
     <row r="22" spans="1:3" ht="20" customHeight="1">
       <c r="A22" t="s">
-        <v>25</v>
-      </c>
-      <c r="B22" t="s">
-        <v>34</v>
+        <v>11</v>
+      </c>
+      <c r="B22" s="5" t="s">
+        <v>32</v>
       </c>
       <c r="C22">
         <v>85</v>
@@ -1390,10 +1311,10 @@
     </row>
     <row r="23" spans="1:3" ht="20" customHeight="1">
       <c r="A23" t="s">
-        <v>25</v>
-      </c>
-      <c r="B23" t="s">
-        <v>37</v>
+        <v>11</v>
+      </c>
+      <c r="B23" s="6" t="s">
+        <v>33</v>
       </c>
       <c r="C23">
         <v>60</v>
@@ -1401,10 +1322,10 @@
     </row>
     <row r="24" spans="1:3" ht="20" customHeight="1">
       <c r="A24" t="s">
-        <v>25</v>
-      </c>
-      <c r="B24" t="s">
-        <v>40</v>
+        <v>11</v>
+      </c>
+      <c r="B24" s="5" t="s">
+        <v>34</v>
       </c>
       <c r="C24">
         <v>22</v>
@@ -1412,10 +1333,10 @@
     </row>
     <row r="25" spans="1:3" ht="20" customHeight="1">
       <c r="A25" t="s">
-        <v>25</v>
-      </c>
-      <c r="B25" t="s">
-        <v>43</v>
+        <v>11</v>
+      </c>
+      <c r="B25" s="6" t="s">
+        <v>35</v>
       </c>
       <c r="C25">
         <v>22</v>
@@ -1423,10 +1344,10 @@
     </row>
     <row r="26" spans="1:3" ht="20" customHeight="1">
       <c r="A26" t="s">
-        <v>25</v>
-      </c>
-      <c r="B26" t="s">
-        <v>45</v>
+        <v>11</v>
+      </c>
+      <c r="B26" s="5" t="s">
+        <v>36</v>
       </c>
       <c r="C26">
         <v>55</v>
@@ -1434,10 +1355,10 @@
     </row>
     <row r="27" spans="1:3" ht="20" customHeight="1">
       <c r="A27" t="s">
-        <v>27</v>
-      </c>
-      <c r="B27" t="s">
-        <v>34</v>
+        <v>12</v>
+      </c>
+      <c r="B27" s="5" t="s">
+        <v>32</v>
       </c>
       <c r="C27">
         <v>120</v>
@@ -1445,10 +1366,10 @@
     </row>
     <row r="28" spans="1:3" ht="20" customHeight="1">
       <c r="A28" t="s">
-        <v>27</v>
-      </c>
-      <c r="B28" t="s">
-        <v>37</v>
+        <v>12</v>
+      </c>
+      <c r="B28" s="6" t="s">
+        <v>33</v>
       </c>
       <c r="C28">
         <v>95</v>
@@ -1456,10 +1377,10 @@
     </row>
     <row r="29" spans="1:3" ht="20" customHeight="1">
       <c r="A29" t="s">
-        <v>27</v>
-      </c>
-      <c r="B29" t="s">
-        <v>40</v>
+        <v>12</v>
+      </c>
+      <c r="B29" s="5" t="s">
+        <v>34</v>
       </c>
       <c r="C29">
         <v>38</v>
@@ -1467,10 +1388,10 @@
     </row>
     <row r="30" spans="1:3" ht="20" customHeight="1">
       <c r="A30" t="s">
-        <v>27</v>
-      </c>
-      <c r="B30" t="s">
-        <v>43</v>
+        <v>12</v>
+      </c>
+      <c r="B30" s="6" t="s">
+        <v>35</v>
       </c>
       <c r="C30">
         <v>32</v>
@@ -1478,10 +1399,10 @@
     </row>
     <row r="31" spans="1:3" ht="20" customHeight="1">
       <c r="A31" t="s">
-        <v>27</v>
-      </c>
-      <c r="B31" t="s">
-        <v>45</v>
+        <v>12</v>
+      </c>
+      <c r="B31" s="5" t="s">
+        <v>36</v>
       </c>
       <c r="C31">
         <v>80</v>

</xml_diff>